<commit_message>
Formatacao do excel. Ok
</commit_message>
<xml_diff>
--- a/New folder/Cube_finish.xlsx
+++ b/New folder/Cube_finish.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Warley Souza\Music\read_excel\New folder\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58272CEE-7658-4D92-BC41-C2DD15DF7161}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCF7894C-7643-4911-A303-8B57ADB94F75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1712" uniqueCount="878">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1708" uniqueCount="877">
   <si>
     <t>Cube</t>
   </si>
@@ -2165,9 +2165,6 @@
   </si>
   <si>
     <t>87A</t>
-  </si>
-  <si>
-    <t>07/02//2022</t>
   </si>
   <si>
     <t>Second Floor Walls(E)(6-11)</t>
@@ -2662,7 +2659,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -2713,12 +2710,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3023,6 +3021,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J581"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="18.109375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
@@ -13596,11 +13597,11 @@
       <c r="A485" t="s">
         <v>714</v>
       </c>
-      <c r="B485" t="s">
+      <c r="B485" s="3">
+        <v>44599</v>
+      </c>
+      <c r="C485" t="s">
         <v>715</v>
-      </c>
-      <c r="C485" t="s">
-        <v>716</v>
       </c>
       <c r="D485" s="2">
         <v>44608</v>
@@ -13609,18 +13610,18 @@
         <v>2310</v>
       </c>
       <c r="F485" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
     </row>
     <row r="486" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A486" t="s">
+        <v>717</v>
+      </c>
+      <c r="B486" s="3">
+        <v>44599</v>
+      </c>
+      <c r="C486" t="s">
         <v>718</v>
-      </c>
-      <c r="B486" t="s">
-        <v>715</v>
-      </c>
-      <c r="C486" t="s">
-        <v>719</v>
       </c>
       <c r="D486" s="2">
         <v>44627</v>
@@ -13634,13 +13635,13 @@
     </row>
     <row r="487" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A487" t="s">
+        <v>719</v>
+      </c>
+      <c r="B487" s="3">
+        <v>44599</v>
+      </c>
+      <c r="C487" t="s">
         <v>720</v>
-      </c>
-      <c r="B487" t="s">
-        <v>715</v>
-      </c>
-      <c r="C487" t="s">
-        <v>721</v>
       </c>
       <c r="D487" s="2">
         <v>44627</v>
@@ -13654,24 +13655,24 @@
     </row>
     <row r="488" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A488" t="s">
+        <v>721</v>
+      </c>
+      <c r="B488" s="3">
+        <v>44599</v>
+      </c>
+      <c r="C488" t="s">
         <v>722</v>
-      </c>
-      <c r="B488" t="s">
-        <v>715</v>
-      </c>
-      <c r="C488" t="s">
-        <v>723</v>
       </c>
     </row>
     <row r="489" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A489" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="B489" s="2">
         <v>44600</v>
       </c>
       <c r="C489" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="D489" s="2">
         <v>44608</v>
@@ -13680,18 +13681,18 @@
         <v>2350</v>
       </c>
       <c r="F489" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="490" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A490" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="B490" s="2">
         <v>44600</v>
       </c>
       <c r="C490" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="D490" s="2">
         <v>44628</v>
@@ -13705,13 +13706,13 @@
     </row>
     <row r="491" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A491" t="s">
-        <v>728</v>
+        <v>727</v>
       </c>
       <c r="B491" s="2">
         <v>44600</v>
       </c>
       <c r="C491" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="D491" s="2">
         <v>44628</v>
@@ -13725,24 +13726,24 @@
     </row>
     <row r="492" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A492" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="B492" s="2">
         <v>44600</v>
       </c>
       <c r="C492" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
     </row>
     <row r="493" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A493" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
       <c r="B493" s="2">
         <v>44600</v>
       </c>
       <c r="C493" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
       <c r="D493" s="2">
         <v>44608</v>
@@ -13751,18 +13752,18 @@
         <v>2360</v>
       </c>
       <c r="F493" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
     </row>
     <row r="494" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A494" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="B494" s="2">
         <v>44600</v>
       </c>
       <c r="C494" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="D494" s="2">
         <v>44628</v>
@@ -13776,13 +13777,13 @@
     </row>
     <row r="495" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A495" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="B495" s="2">
         <v>44600</v>
       </c>
       <c r="C495" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="D495" s="2">
         <v>44628</v>
@@ -13796,24 +13797,24 @@
     </row>
     <row r="496" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A496" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="B496" s="2">
         <v>44600</v>
       </c>
       <c r="C496" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
     </row>
     <row r="497" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A497" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
       <c r="B497" s="2">
         <v>44601</v>
       </c>
       <c r="C497" t="s">
-        <v>739</v>
+        <v>738</v>
       </c>
       <c r="D497" s="2">
         <v>44608</v>
@@ -13822,69 +13823,69 @@
         <v>2390</v>
       </c>
       <c r="F497" t="s">
-        <v>740</v>
+        <v>739</v>
       </c>
     </row>
     <row r="498" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A498" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
       <c r="B498" s="2">
         <v>44601</v>
       </c>
       <c r="C498" t="s">
+        <v>741</v>
+      </c>
+      <c r="D498" t="s">
         <v>742</v>
       </c>
-      <c r="D498" t="s">
+      <c r="E498" t="s">
         <v>743</v>
       </c>
-      <c r="E498" t="s">
+      <c r="H498" t="s">
         <v>744</v>
-      </c>
-      <c r="H498" t="s">
-        <v>745</v>
       </c>
     </row>
     <row r="499" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A499" t="s">
-        <v>746</v>
+        <v>745</v>
       </c>
       <c r="B499" s="2">
         <v>44601</v>
       </c>
       <c r="C499" t="s">
+        <v>746</v>
+      </c>
+      <c r="D499" t="s">
+        <v>742</v>
+      </c>
+      <c r="E499" t="s">
         <v>747</v>
       </c>
-      <c r="D499" t="s">
-        <v>743</v>
-      </c>
-      <c r="E499" t="s">
+      <c r="H499" t="s">
         <v>748</v>
-      </c>
-      <c r="H499" t="s">
-        <v>749</v>
       </c>
     </row>
     <row r="500" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A500" t="s">
-        <v>750</v>
+        <v>749</v>
       </c>
       <c r="B500" s="2">
         <v>44601</v>
       </c>
       <c r="C500" t="s">
-        <v>747</v>
+        <v>746</v>
       </c>
     </row>
     <row r="501" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A501" t="s">
-        <v>751</v>
+        <v>750</v>
       </c>
       <c r="B501" s="2">
         <v>44602</v>
       </c>
       <c r="C501" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="D501" s="2">
         <v>44616</v>
@@ -13898,64 +13899,64 @@
     </row>
     <row r="502" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A502" t="s">
-        <v>753</v>
+        <v>752</v>
       </c>
       <c r="B502" s="2">
         <v>44602</v>
       </c>
       <c r="C502" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="D502" t="s">
         <v>598</v>
       </c>
       <c r="E502" t="s">
+        <v>753</v>
+      </c>
+      <c r="H502" t="s">
         <v>754</v>
-      </c>
-      <c r="H502" t="s">
-        <v>755</v>
       </c>
     </row>
     <row r="503" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A503" t="s">
-        <v>756</v>
+        <v>755</v>
       </c>
       <c r="B503" s="2">
         <v>44602</v>
       </c>
       <c r="C503" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="D503" t="s">
         <v>598</v>
       </c>
       <c r="E503" t="s">
-        <v>754</v>
+        <v>753</v>
       </c>
       <c r="H503" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
     </row>
     <row r="504" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A504" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
       <c r="B504" s="2">
         <v>44602</v>
       </c>
       <c r="C504" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
     </row>
     <row r="505" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A505" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="B505" s="2">
         <v>44603</v>
       </c>
       <c r="C505" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
       <c r="D505" s="2">
         <v>44615</v>
@@ -13969,13 +13970,13 @@
     </row>
     <row r="506" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A506" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="B506" s="2">
         <v>44603</v>
       </c>
       <c r="C506" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
       <c r="D506" s="2">
         <v>44617</v>
@@ -13989,13 +13990,13 @@
     </row>
     <row r="507" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A507" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
       <c r="B507" s="2">
         <v>44603</v>
       </c>
       <c r="C507" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
       <c r="D507" t="s">
         <v>608</v>
@@ -14009,13 +14010,13 @@
     </row>
     <row r="508" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A508" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
       <c r="B508" s="2">
         <v>44603</v>
       </c>
       <c r="C508" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
       <c r="D508" t="s">
         <v>608</v>
@@ -14029,24 +14030,24 @@
     </row>
     <row r="509" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A509" t="s">
-        <v>763</v>
+        <v>762</v>
       </c>
       <c r="B509" s="2">
         <v>44603</v>
       </c>
       <c r="C509" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
     </row>
     <row r="510" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A510" t="s">
-        <v>764</v>
+        <v>763</v>
       </c>
       <c r="B510" s="2">
         <v>44606</v>
       </c>
       <c r="C510" t="s">
-        <v>765</v>
+        <v>764</v>
       </c>
       <c r="D510" s="2">
         <v>44615</v>
@@ -14060,13 +14061,13 @@
     </row>
     <row r="511" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A511" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="B511" s="2">
         <v>44606</v>
       </c>
       <c r="C511" t="s">
-        <v>765</v>
+        <v>764</v>
       </c>
       <c r="D511" t="s">
         <v>617</v>
@@ -14080,13 +14081,13 @@
     </row>
     <row r="512" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A512" t="s">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="B512" s="2">
         <v>44606</v>
       </c>
       <c r="C512" t="s">
-        <v>765</v>
+        <v>764</v>
       </c>
       <c r="D512" t="s">
         <v>617</v>
@@ -14100,35 +14101,35 @@
     </row>
     <row r="513" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A513" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
       <c r="B513" s="2">
         <v>44606</v>
       </c>
       <c r="C513" t="s">
-        <v>765</v>
+        <v>764</v>
       </c>
     </row>
     <row r="514" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A514" t="s">
-        <v>769</v>
+        <v>768</v>
       </c>
       <c r="B514" s="2">
         <v>44606</v>
       </c>
       <c r="C514" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
     </row>
     <row r="515" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A515" t="s">
-        <v>771</v>
+        <v>770</v>
       </c>
       <c r="B515" s="2">
         <v>44606</v>
       </c>
       <c r="C515" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="D515" t="s">
         <v>617</v>
@@ -14142,13 +14143,13 @@
     </row>
     <row r="516" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A516" t="s">
-        <v>772</v>
+        <v>771</v>
       </c>
       <c r="B516" s="2">
         <v>44606</v>
       </c>
       <c r="C516" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="D516" t="s">
         <v>617</v>
@@ -14162,793 +14163,793 @@
     </row>
     <row r="517" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A517" t="s">
-        <v>773</v>
+        <v>772</v>
       </c>
       <c r="B517" s="2">
         <v>44606</v>
       </c>
       <c r="C517" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
     </row>
     <row r="518" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A518" t="s">
-        <v>774</v>
+        <v>773</v>
       </c>
       <c r="B518" s="2">
         <v>44607</v>
       </c>
       <c r="C518" t="s">
-        <v>775</v>
+        <v>774</v>
       </c>
       <c r="D518" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
       <c r="E518" t="s">
         <v>599</v>
       </c>
       <c r="F518" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
     </row>
     <row r="519" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A519" t="s">
-        <v>777</v>
+        <v>776</v>
       </c>
       <c r="B519" s="2">
         <v>44607</v>
       </c>
       <c r="C519" t="s">
-        <v>775</v>
+        <v>774</v>
       </c>
       <c r="D519" t="s">
-        <v>778</v>
+        <v>777</v>
       </c>
       <c r="E519" t="s">
         <v>609</v>
       </c>
       <c r="H519" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
     </row>
     <row r="520" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A520" t="s">
-        <v>780</v>
+        <v>779</v>
       </c>
       <c r="B520" s="2">
         <v>44607</v>
       </c>
       <c r="C520" t="s">
-        <v>775</v>
+        <v>774</v>
       </c>
       <c r="D520" t="s">
-        <v>778</v>
+        <v>777</v>
       </c>
       <c r="E520" t="s">
         <v>599</v>
       </c>
       <c r="H520" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
     </row>
     <row r="521" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A521" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="B521" s="2">
         <v>44607</v>
       </c>
       <c r="C521" t="s">
-        <v>775</v>
+        <v>774</v>
       </c>
     </row>
     <row r="522" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A522" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="B522" s="2">
         <v>44608</v>
       </c>
       <c r="C522" t="s">
+        <v>783</v>
+      </c>
+      <c r="D522" t="s">
+        <v>742</v>
+      </c>
+      <c r="E522" t="s">
+        <v>753</v>
+      </c>
+      <c r="F522" t="s">
         <v>784</v>
-      </c>
-      <c r="D522" t="s">
-        <v>743</v>
-      </c>
-      <c r="E522" t="s">
-        <v>754</v>
-      </c>
-      <c r="F522" t="s">
-        <v>785</v>
       </c>
     </row>
     <row r="523" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A523" t="s">
-        <v>786</v>
+        <v>785</v>
       </c>
       <c r="B523" s="2">
         <v>44608</v>
       </c>
       <c r="C523" t="s">
-        <v>784</v>
+        <v>783</v>
       </c>
     </row>
     <row r="524" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A524" t="s">
-        <v>787</v>
+        <v>786</v>
       </c>
       <c r="B524" s="2">
         <v>44608</v>
       </c>
       <c r="C524" t="s">
-        <v>784</v>
+        <v>783</v>
       </c>
     </row>
     <row r="525" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A525" t="s">
-        <v>788</v>
+        <v>787</v>
       </c>
       <c r="B525" s="2">
         <v>44608</v>
       </c>
       <c r="C525" t="s">
-        <v>784</v>
+        <v>783</v>
       </c>
     </row>
     <row r="526" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A526" t="s">
-        <v>789</v>
+        <v>788</v>
       </c>
       <c r="B526" s="2">
         <v>44609</v>
       </c>
       <c r="C526" t="s">
+        <v>789</v>
+      </c>
+      <c r="D526" t="s">
+        <v>742</v>
+      </c>
+      <c r="E526" t="s">
+        <v>753</v>
+      </c>
+      <c r="F526" t="s">
         <v>790</v>
-      </c>
-      <c r="D526" t="s">
-        <v>743</v>
-      </c>
-      <c r="E526" t="s">
-        <v>754</v>
-      </c>
-      <c r="F526" t="s">
-        <v>791</v>
       </c>
     </row>
     <row r="527" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A527" t="s">
-        <v>792</v>
+        <v>791</v>
       </c>
       <c r="B527" s="2">
         <v>44609</v>
       </c>
       <c r="C527" t="s">
-        <v>790</v>
+        <v>789</v>
       </c>
     </row>
     <row r="528" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A528" t="s">
-        <v>793</v>
+        <v>792</v>
       </c>
       <c r="B528" s="2">
         <v>44609</v>
       </c>
       <c r="C528" t="s">
-        <v>790</v>
+        <v>789</v>
       </c>
     </row>
     <row r="529" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A529" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
       <c r="B529" s="2">
         <v>44609</v>
       </c>
       <c r="C529" t="s">
-        <v>790</v>
+        <v>789</v>
       </c>
     </row>
     <row r="530" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A530" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
       <c r="B530" s="2">
         <v>44610</v>
       </c>
       <c r="C530" t="s">
+        <v>795</v>
+      </c>
+      <c r="D530" t="s">
+        <v>742</v>
+      </c>
+      <c r="E530" t="s">
+        <v>753</v>
+      </c>
+      <c r="F530" t="s">
         <v>796</v>
-      </c>
-      <c r="D530" t="s">
-        <v>743</v>
-      </c>
-      <c r="E530" t="s">
-        <v>754</v>
-      </c>
-      <c r="F530" t="s">
-        <v>797</v>
       </c>
     </row>
     <row r="531" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A531" t="s">
-        <v>798</v>
+        <v>797</v>
       </c>
       <c r="B531" s="2">
         <v>44610</v>
       </c>
       <c r="C531" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
     </row>
     <row r="532" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A532" t="s">
-        <v>799</v>
+        <v>798</v>
       </c>
       <c r="B532" s="2">
         <v>44610</v>
       </c>
       <c r="C532" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
     </row>
     <row r="533" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A533" t="s">
-        <v>800</v>
+        <v>799</v>
       </c>
       <c r="B533" s="2">
         <v>44610</v>
       </c>
       <c r="C533" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
     </row>
     <row r="534" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A534" t="s">
-        <v>801</v>
+        <v>800</v>
       </c>
       <c r="B534" s="2">
         <v>44613</v>
       </c>
       <c r="C534" t="s">
+        <v>801</v>
+      </c>
+      <c r="D534" t="s">
+        <v>742</v>
+      </c>
+      <c r="E534" t="s">
         <v>802</v>
       </c>
-      <c r="D534" t="s">
-        <v>743</v>
-      </c>
-      <c r="E534" t="s">
+      <c r="F534" t="s">
         <v>803</v>
-      </c>
-      <c r="F534" t="s">
-        <v>804</v>
       </c>
     </row>
     <row r="535" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A535" t="s">
-        <v>805</v>
+        <v>804</v>
       </c>
       <c r="B535" s="2">
         <v>44613</v>
       </c>
       <c r="C535" t="s">
-        <v>802</v>
+        <v>801</v>
       </c>
     </row>
     <row r="536" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A536" t="s">
-        <v>806</v>
+        <v>805</v>
       </c>
       <c r="B536" s="2">
         <v>44613</v>
       </c>
       <c r="C536" t="s">
-        <v>802</v>
+        <v>801</v>
       </c>
     </row>
     <row r="537" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A537" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="B537" s="2">
         <v>44613</v>
       </c>
       <c r="C537" t="s">
-        <v>802</v>
+        <v>801</v>
       </c>
     </row>
     <row r="538" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A538" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="B538" s="2">
         <v>44614</v>
       </c>
       <c r="C538" t="s">
+        <v>808</v>
+      </c>
+      <c r="D538" t="s">
+        <v>742</v>
+      </c>
+      <c r="E538" t="s">
         <v>809</v>
       </c>
-      <c r="D538" t="s">
-        <v>743</v>
-      </c>
-      <c r="E538" t="s">
+      <c r="F538" t="s">
         <v>810</v>
-      </c>
-      <c r="F538" t="s">
-        <v>811</v>
       </c>
     </row>
     <row r="539" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A539" t="s">
-        <v>812</v>
+        <v>811</v>
       </c>
       <c r="B539" s="2">
         <v>44614</v>
       </c>
       <c r="C539" t="s">
-        <v>809</v>
+        <v>808</v>
       </c>
     </row>
     <row r="540" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A540" t="s">
-        <v>813</v>
+        <v>812</v>
       </c>
       <c r="B540" s="2">
         <v>44614</v>
       </c>
       <c r="C540" t="s">
-        <v>809</v>
+        <v>808</v>
       </c>
     </row>
     <row r="541" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A541" t="s">
-        <v>814</v>
+        <v>813</v>
       </c>
       <c r="B541" s="2">
         <v>44614</v>
       </c>
       <c r="C541" t="s">
-        <v>809</v>
+        <v>808</v>
       </c>
     </row>
     <row r="542" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A542" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="B542" s="2">
         <v>44614</v>
       </c>
       <c r="C542" t="s">
+        <v>815</v>
+      </c>
+      <c r="D542" t="s">
+        <v>742</v>
+      </c>
+      <c r="E542" t="s">
+        <v>743</v>
+      </c>
+      <c r="F542" t="s">
         <v>816</v>
-      </c>
-      <c r="D542" t="s">
-        <v>743</v>
-      </c>
-      <c r="E542" t="s">
-        <v>744</v>
-      </c>
-      <c r="F542" t="s">
-        <v>817</v>
       </c>
     </row>
     <row r="543" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A543" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
       <c r="B543" s="2">
         <v>44614</v>
       </c>
       <c r="C543" t="s">
-        <v>816</v>
+        <v>815</v>
       </c>
     </row>
     <row r="544" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A544" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="B544" s="2">
         <v>44614</v>
       </c>
       <c r="C544" t="s">
-        <v>816</v>
+        <v>815</v>
       </c>
     </row>
     <row r="545" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A545" t="s">
-        <v>820</v>
+        <v>819</v>
       </c>
       <c r="B545" s="2">
         <v>44614</v>
       </c>
       <c r="C545" t="s">
-        <v>816</v>
+        <v>815</v>
       </c>
     </row>
     <row r="546" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A546" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="B546" s="2">
         <v>44615</v>
       </c>
       <c r="C546" t="s">
+        <v>821</v>
+      </c>
+      <c r="D546" t="s">
+        <v>742</v>
+      </c>
+      <c r="E546" t="s">
+        <v>802</v>
+      </c>
+      <c r="G546" t="s">
         <v>822</v>
-      </c>
-      <c r="D546" t="s">
-        <v>743</v>
-      </c>
-      <c r="E546" t="s">
-        <v>803</v>
-      </c>
-      <c r="G546" t="s">
-        <v>823</v>
       </c>
     </row>
     <row r="547" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A547" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
       <c r="B547" s="2">
         <v>44615</v>
       </c>
       <c r="C547" t="s">
-        <v>822</v>
+        <v>821</v>
       </c>
     </row>
     <row r="548" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A548" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
       <c r="B548" s="2">
         <v>44615</v>
       </c>
       <c r="C548" t="s">
-        <v>822</v>
+        <v>821</v>
       </c>
     </row>
     <row r="549" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A549" t="s">
-        <v>826</v>
+        <v>825</v>
       </c>
       <c r="B549" s="2">
         <v>44615</v>
       </c>
       <c r="C549" t="s">
-        <v>822</v>
+        <v>821</v>
       </c>
     </row>
     <row r="550" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A550" t="s">
-        <v>827</v>
+        <v>826</v>
       </c>
       <c r="B550" s="2">
         <v>44616</v>
       </c>
       <c r="C550" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
       <c r="D550" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
       <c r="E550" t="s">
         <v>609</v>
       </c>
       <c r="F550" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
     </row>
     <row r="551" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A551" t="s">
-        <v>830</v>
+        <v>829</v>
       </c>
       <c r="B551" s="2">
         <v>44616</v>
       </c>
       <c r="C551" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
     </row>
     <row r="552" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A552" t="s">
-        <v>831</v>
+        <v>830</v>
       </c>
       <c r="B552" s="2">
         <v>44616</v>
       </c>
       <c r="C552" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
       <c r="D552" t="s">
         <v>617</v>
       </c>
       <c r="E552" t="s">
+        <v>831</v>
+      </c>
+      <c r="H552" t="s">
         <v>832</v>
-      </c>
-      <c r="H552" t="s">
-        <v>833</v>
       </c>
     </row>
     <row r="553" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A553" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="B553" s="2">
         <v>44616</v>
       </c>
       <c r="C553" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
     </row>
     <row r="554" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A554" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="B554" s="2">
         <v>44617</v>
       </c>
       <c r="C554" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="D554" t="s">
         <v>608</v>
       </c>
       <c r="E554" t="s">
+        <v>836</v>
+      </c>
+      <c r="G554" t="s">
         <v>837</v>
-      </c>
-      <c r="G554" t="s">
-        <v>838</v>
       </c>
     </row>
     <row r="555" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A555" t="s">
-        <v>839</v>
+        <v>838</v>
       </c>
       <c r="B555" s="2">
         <v>44617</v>
       </c>
       <c r="C555" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
     </row>
     <row r="556" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A556" t="s">
-        <v>840</v>
+        <v>839</v>
       </c>
       <c r="B556" s="2">
         <v>44617</v>
       </c>
       <c r="C556" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
     </row>
     <row r="557" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A557" t="s">
-        <v>841</v>
+        <v>840</v>
       </c>
       <c r="B557" s="2">
         <v>44617</v>
       </c>
       <c r="C557" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
     </row>
     <row r="558" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A558" t="s">
-        <v>842</v>
+        <v>841</v>
       </c>
       <c r="B558" s="2">
         <v>44620</v>
       </c>
       <c r="C558" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="D558" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
       <c r="E558" t="s">
         <v>609</v>
       </c>
       <c r="F558" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
     </row>
     <row r="559" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A559" t="s">
-        <v>845</v>
+        <v>844</v>
       </c>
       <c r="B559" s="2">
         <v>44620</v>
       </c>
       <c r="C559" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
     </row>
     <row r="560" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A560" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
       <c r="B560" s="2">
         <v>44620</v>
       </c>
       <c r="C560" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
     </row>
     <row r="561" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A561" t="s">
-        <v>847</v>
+        <v>846</v>
       </c>
       <c r="B561" s="2">
         <v>44620</v>
       </c>
       <c r="C561" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
     </row>
     <row r="562" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A562" t="s">
-        <v>848</v>
+        <v>847</v>
       </c>
       <c r="B562" s="2">
         <v>44620</v>
       </c>
       <c r="C562" t="s">
+        <v>848</v>
+      </c>
+      <c r="D562" t="s">
+        <v>742</v>
+      </c>
+      <c r="E562" t="s">
+        <v>802</v>
+      </c>
+      <c r="F562" t="s">
         <v>849</v>
-      </c>
-      <c r="D562" t="s">
-        <v>743</v>
-      </c>
-      <c r="E562" t="s">
-        <v>803</v>
-      </c>
-      <c r="F562" t="s">
-        <v>850</v>
       </c>
     </row>
     <row r="563" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A563" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="B563" s="2">
         <v>44620</v>
       </c>
       <c r="C563" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
     </row>
     <row r="564" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A564" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="B564" s="2">
         <v>44620</v>
       </c>
       <c r="C564" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
     </row>
     <row r="565" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A565" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
       <c r="B565" s="2">
         <v>44620</v>
       </c>
       <c r="C565" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
     </row>
     <row r="566" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A566" t="s">
-        <v>854</v>
+        <v>853</v>
       </c>
       <c r="B566" s="2">
         <v>44621</v>
       </c>
       <c r="C566" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="D566" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
       <c r="E566" t="s">
         <v>599</v>
       </c>
       <c r="F566" t="s">
-        <v>856</v>
+        <v>855</v>
       </c>
     </row>
     <row r="567" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A567" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
       <c r="B567" s="2">
         <v>44621</v>
       </c>
       <c r="C567" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
     </row>
     <row r="568" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A568" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
       <c r="B568" s="2">
         <v>44621</v>
       </c>
       <c r="C568" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
     </row>
     <row r="569" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A569" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
       <c r="B569" s="2">
         <v>44621</v>
       </c>
       <c r="C569" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
     </row>
     <row r="570" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A570" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
       <c r="B570" s="2">
         <v>44622</v>
       </c>
       <c r="C570" t="s">
-        <v>861</v>
+        <v>860</v>
       </c>
       <c r="D570" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
       <c r="E570" t="s">
         <v>609</v>
       </c>
       <c r="F570" t="s">
-        <v>862</v>
+        <v>861</v>
       </c>
     </row>
     <row r="571" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A571" t="s">
-        <v>863</v>
+        <v>862</v>
       </c>
       <c r="B571" s="2">
         <v>44622</v>
       </c>
       <c r="C571" t="s">
-        <v>861</v>
+        <v>860</v>
       </c>
     </row>
     <row r="572" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A572" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
       <c r="B572" s="2">
         <v>44622</v>
       </c>
       <c r="C572" t="s">
-        <v>861</v>
+        <v>860</v>
       </c>
     </row>
     <row r="573" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A573" t="s">
-        <v>865</v>
+        <v>864</v>
       </c>
       <c r="B573" s="2">
         <v>44622</v>
       </c>
       <c r="C573" t="s">
-        <v>861</v>
+        <v>860</v>
       </c>
     </row>
     <row r="574" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A574" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
       <c r="B574" s="2">
         <v>44623</v>
       </c>
       <c r="C574" t="s">
-        <v>867</v>
+        <v>866</v>
       </c>
       <c r="D574" t="s">
         <v>598</v>
@@ -14957,93 +14958,93 @@
         <v>599</v>
       </c>
       <c r="F574" t="s">
-        <v>868</v>
+        <v>867</v>
       </c>
     </row>
     <row r="575" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A575" t="s">
-        <v>869</v>
+        <v>868</v>
       </c>
       <c r="B575" s="2">
         <v>44623</v>
       </c>
       <c r="C575" t="s">
-        <v>867</v>
+        <v>866</v>
       </c>
     </row>
     <row r="576" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A576" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
       <c r="B576" s="2">
         <v>44623</v>
       </c>
       <c r="C576" t="s">
-        <v>867</v>
+        <v>866</v>
       </c>
     </row>
     <row r="577" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A577" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
       <c r="B577" s="2">
         <v>44623</v>
       </c>
       <c r="C577" t="s">
-        <v>867</v>
+        <v>866</v>
       </c>
     </row>
     <row r="578" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A578" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="B578" s="2">
         <v>44624</v>
       </c>
       <c r="C578" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="D578" t="s">
         <v>608</v>
       </c>
       <c r="E578" t="s">
-        <v>754</v>
+        <v>753</v>
       </c>
       <c r="F578" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
     </row>
     <row r="579" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A579" t="s">
-        <v>875</v>
+        <v>874</v>
       </c>
       <c r="B579" s="2">
         <v>44624</v>
       </c>
       <c r="C579" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
     </row>
     <row r="580" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A580" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="B580" s="2">
         <v>44624</v>
       </c>
       <c r="C580" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
     </row>
     <row r="581" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A581" t="s">
-        <v>877</v>
+        <v>876</v>
       </c>
       <c r="B581" s="2">
         <v>44624</v>
       </c>
       <c r="C581" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
     </row>
   </sheetData>

</xml_diff>